<commit_message>
Refine UART VIP checks, frame configuration and start timing
</commit_message>
<xml_diff>
--- a/Vplan.xlsx
+++ b/Vplan.xlsx
@@ -132,19 +132,19 @@
       </c>
       <c r="B4" t="inlineStr" s="0">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" t="inlineStr" s="0">
         <is>
-          <t>DUT cases / checker self-test</t>
+          <t>DUT cases / checker self-tests</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="0">
         <is>
-          <t>28 / 1</t>
+          <t>28 / 2</t>
         </is>
       </c>
     </row>
@@ -156,7 +156,7 @@
       </c>
       <c r="B6" t="inlineStr" s="0">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
     </row>
@@ -168,7 +168,7 @@
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t>23 / 10 / 0</t>
+          <t>24 / 10 / 0</t>
         </is>
       </c>
     </row>
@@ -336,7 +336,7 @@
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t>PASS=3 FAIL=1 UNKNOWN=0</t>
+          <t>PASS=4 FAIL=1 UNKNOWN=0</t>
         </is>
       </c>
     </row>
@@ -370,7 +370,7 @@
       </c>
       <c r="B1" t="inlineStr" s="0">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
     </row>
@@ -382,7 +382,7 @@
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -2283,8 +2283,70 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="64" customHeight="1">
+      <c r="A37" t="inlineStr" s="0">
+        <is>
+          <t>SYS-05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr" s="0">
+        <is>
+          <t>9. Integration and checker</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="0">
+        <is>
+          <t>Standalone VIP loopback: constrained frame configuration, initial idle delay, contiguous frames, parity and stop errors</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr" s="0">
+        <is>
+          <t>uart_vip_contract_test</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr" s="0">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr" s="0">
+        <is>
+          <t>No scoreboard: monitor reports both directions; exact caught-error counts; pin timing checks; 100 constrained configurations</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr" s="0">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr" s="2">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr" s="0">
+        <is>
+          <t>Checker self-test; isolated pins, not a DUT compliance result</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr" s="0">
+        <is>
+          <t>UART VIP review notes; UVM GUIDE 3</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr" s="0">
+        <is>
+          <t>seed=1 PASS sim/log/uart_vip_contract_test_1.log</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:L36"/>
+  <autoFilter ref="A7:L37"/>
 </worksheet>
 </file>
 
@@ -2439,7 +2501,7 @@
       </c>
       <c r="F4" t="inlineStr" s="0">
         <is>
-          <t>make -C sim run TESTNAME=uart_rx_13x_div2_test SEED=1 COV=ON (expected nonzero). Also observed in duplex seeds 2–5.</t>
+          <t>make -C sim run TESTNAME=uart_rx_13x_div2_test SEED=1 COV=ON (expected nonzero). Also observed in current duplex seeds 2, 3, 4, 5.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr" s="0">
@@ -2690,7 +2752,7 @@
       </c>
       <c r="B14" t="inlineStr" s="0">
         <is>
-          <t>33 completed runs</t>
+          <t>34 completed runs</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="0">

</xml_diff>